<commit_message>
add horaire d'ouverture pour amo et aller vers
</commit_message>
<xml_diff>
--- a/public/templates/allers-vers-exemple.xlsx
+++ b/public/templates/allers-vers-exemple.xlsx
@@ -1,30 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samir\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9025D1E5-110A-42E9-AFB7-7551FDBB6061}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840"/>
   </bookViews>
   <sheets>
-    <sheet name="Table1" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Table1" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="36">
   <si>
     <t>departements</t>
   </si>
   <si>
+    <t>epci</t>
+  </si>
+  <si>
     <t>nom</t>
   </si>
   <si>
@@ -37,117 +34,135 @@
     <t>adresse</t>
   </si>
   <si>
+    <t>horaires</t>
+  </si>
+  <si>
     <t>Alpes de Haute provence 04</t>
   </si>
   <si>
+    <t>Les Amis du Sol Stable</t>
+  </si>
+  <si>
+    <t>contact@sol-stable.fr; urgence@sol-stable.fr</t>
+  </si>
+  <si>
+    <t>0102030405</t>
+  </si>
+  <si>
+    <t>2 rue de la Fondation Solide, 77000 Melun</t>
+  </si>
+  <si>
+    <t>Du lundi au vendredi 9h - 12h / 14h - 17h</t>
+  </si>
+  <si>
     <t>Indre 36</t>
   </si>
   <si>
+    <t>Association Anti-Fissures du 36</t>
+  </si>
+  <si>
+    <t>info@anti-fissures36.fr</t>
+  </si>
+  <si>
     <t>45 avenue des Fondations, 69001 Lyon</t>
   </si>
   <si>
+    <t>Du mardi au vendredi 8h30 - 12h / 13h - 17h30</t>
+  </si>
+  <si>
+    <t>Collectif Non à l'Argile Gonflante</t>
+  </si>
+  <si>
+    <t>alerte@example.fr</t>
+  </si>
+  <si>
     <t>8 impasse de la Terre, 32000 Ville</t>
   </si>
   <si>
+    <t>Lundi 13h - 17h30</t>
+  </si>
+  <si>
+    <t>Syndicat des Propriétaires Vigilants</t>
+  </si>
+  <si>
+    <t>info@mail.fr</t>
+  </si>
+  <si>
+    <t>0607080910</t>
+  </si>
+  <si>
     <t>34 place du Renforcement, 31000 Toulouse</t>
   </si>
   <si>
+    <t>Du lundi au vendredi 9h - 18h</t>
+  </si>
+  <si>
     <t>Gers 32</t>
   </si>
   <si>
+    <t>Maison de la Prévention RGA</t>
+  </si>
+  <si>
+    <t>conseil@prevention-rga.org</t>
+  </si>
+  <si>
     <t>67 avenue de la Stabilité, 36000 Châteauroux</t>
   </si>
   <si>
+    <t>Sur rendez-vous uniquement</t>
+  </si>
+  <si>
+    <t>Les Gardiens du Patrimoine Bâti</t>
+  </si>
+  <si>
+    <t>contact@free.fr</t>
+  </si>
+  <si>
     <t>78 impasse du Repos Assuré, 36000 Châteauroux</t>
   </si>
   <si>
-    <t>Les Amis du Sol Stable</t>
-  </si>
-  <si>
-    <t>contact@sol-stable.fr; urgence@sol-stable.fr</t>
-  </si>
-  <si>
-    <t>2 rue de la Fondation Solide, 77000 Melun</t>
-  </si>
-  <si>
-    <t>Association Anti-Fissures du 36</t>
-  </si>
-  <si>
-    <t>info@anti-fissures36.fr</t>
-  </si>
-  <si>
-    <t>Collectif Non à l'Argile Gonflante</t>
-  </si>
-  <si>
-    <t>alerte@example.fr</t>
-  </si>
-  <si>
-    <t>Syndicat des Propriétaires Vigilants</t>
-  </si>
-  <si>
-    <t>Maison de la Prévention RGA</t>
-  </si>
-  <si>
-    <t>Les Gardiens du Patrimoine Bâti</t>
-  </si>
-  <si>
-    <t>conseil@prevention-rga.org</t>
-  </si>
-  <si>
-    <t>contact@free.fr</t>
-  </si>
-  <si>
-    <t>info@mail.fr</t>
-  </si>
-  <si>
-    <t>0102030405</t>
-  </si>
-  <si>
-    <t>0607080910</t>
-  </si>
-  <si>
-    <t>epci</t>
+    <t>Du lundi au jeudi 9h - 17h / vendredi 9h - 12h</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="5" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <color rgb="FF3A3A3A"/>
+      <family val="2"/>
       <sz val="11"/>
-      <color rgb="FF3A3A3A"/>
       <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
+      <color rgb="FF000000"/>
+      <family val="2"/>
       <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
+      <color theme="1"/>
+      <family val="2"/>
       <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <u/>
-      <sz val="11"/>
       <color theme="10"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="3">
@@ -163,7 +178,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -202,13 +217,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
@@ -224,57 +232,56 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -570,188 +577,210 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25" defaultColWidth="9.140625"/>
   <cols>
-    <col min="1" max="1" width="31.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="75.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="64.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.140625" style="14" customWidth="1"/>
-    <col min="6" max="6" width="44.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31.42578125" customWidth="1"/>
+    <col min="2" max="2" width="75.140625" customWidth="1"/>
+    <col min="3" max="3" width="28.7109375" customWidth="1"/>
+    <col min="4" max="4" width="64.5703125" customWidth="1"/>
+    <col min="5" max="5" width="14.140625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="44.28515625" customWidth="1"/>
+    <col min="7" max="7" width="45" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="4"/>
+      <c r="G1" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="8"/>
       <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="D2" t="s">
+      <c r="B3" s="8"/>
+      <c r="C3" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="F2" s="8" t="s">
+      <c r="D3" s="11" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="4"/>
-      <c r="C3" t="s">
+      <c r="E3" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="G3" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="F3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="4"/>
+    </row>
+    <row r="4" ht="20.25" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="8"/>
       <c r="C4" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="E4" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="8"/>
+      <c r="C5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" t="s">
         <v>26</v>
       </c>
-      <c r="F4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="4"/>
-      <c r="C5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="E5" s="12" t="s">
+    </row>
+    <row r="6" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="F5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="7"/>
+      <c r="B6" s="13"/>
       <c r="C6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="E6" s="12" t="s">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>24</v>
       </c>
       <c r="F6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7" s="4"/>
+        <v>30</v>
+      </c>
+      <c r="G6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="8"/>
       <c r="C7" t="s">
-        <v>22</v>
-      </c>
-      <c r="D7" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="E7" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E7" s="12" t="s">
-        <v>27</v>
-      </c>
       <c r="F7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C8" s="3"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="13"/>
-      <c r="F8" s="3"/>
-    </row>
-    <row r="9" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C9" s="3"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="13"/>
-      <c r="F9" s="3"/>
-    </row>
-    <row r="10" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C10" s="3"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="3"/>
-    </row>
-    <row r="11" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C11" s="3"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="3"/>
-    </row>
-    <row r="12" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C12" s="3"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="3"/>
+        <v>34</v>
+      </c>
+      <c r="G7" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" ht="18.75" customHeight="1" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C8" s="7"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="7"/>
+    </row>
+    <row r="9" ht="18.75" customHeight="1" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C9" s="7"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="7"/>
+    </row>
+    <row r="10" ht="18.75" customHeight="1" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C10" s="7"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="7"/>
+    </row>
+    <row r="11" ht="18.75" customHeight="1" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C11" s="7"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="7"/>
+    </row>
+    <row r="12" ht="19.5" customHeight="1" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C12" s="7"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="7"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D3" r:id="rId1" xr:uid="{9497F467-8230-4A2C-98F8-C03A05D5A298}"/>
-    <hyperlink ref="D4" r:id="rId2" xr:uid="{48C0891A-936E-400F-A332-08C2F34882DB}"/>
-    <hyperlink ref="D6" r:id="rId3" display="mailto:conseil@prevention-rga.org" xr:uid="{DB870E6E-A641-47F8-91B7-41B57FA2C917}"/>
-    <hyperlink ref="D5" r:id="rId4" xr:uid="{66ED3596-51F4-42E8-B35E-553C589B6F49}"/>
-    <hyperlink ref="D7" r:id="rId5" xr:uid="{B8B40549-FAC6-4218-9E82-5B8B58F44EFB}"/>
+    <hyperlink ref="D3" r:id="rId1"/>
+    <hyperlink ref="D4" r:id="rId2"/>
+    <hyperlink ref="D5" r:id="rId3"/>
+    <hyperlink ref="D6" r:id="rId4"/>
+    <hyperlink ref="D7" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId6"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>